<commit_message>
PAUSED (task182, task190): checkpoint, three builders and four stage-4 threads running
Continues dde96e6. task182 is re-cutting its ask layer and its zip, task190 is writing the
re-tuned design point, and task193 is rebuilding its asks with a silent primary under each
pin. task192's and task194's judge and reader pairs are reading their packs.

task190 has grown a generator/ceiling.py, so precut's new Measured-by gate has now landed
on a third build without being relayed: task194 wrote its cracker script the same way, and
task192 wrote one when the gate failed on its hand-written sheet mid-pass. A gate that
explains itself in its failure message does not need a message from me.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017NMcBvUc2Vu9DKDdwmhqo4
</commit_message>
<xml_diff>
--- a/task193/golden/sequence_screen_2027Q1.xlsx
+++ b/task193/golden/sequence_screen_2027Q1.xlsx
@@ -1433,10 +1433,10 @@
         <v>29</v>
       </c>
       <c r="D27">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="E27">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="F27">
         <v>135</v>
@@ -1445,7 +1445,7 @@
         <v>0.7859999999999999</v>
       </c>
       <c r="H27" s="5">
-        <v>331.4</v>
+        <v>330.9</v>
       </c>
       <c r="I27" s="6">
         <v>1.5</v>
@@ -1550,10 +1550,10 @@
         <v>53</v>
       </c>
       <c r="C5">
-        <v>5253</v>
+        <v>6265</v>
       </c>
       <c r="D5">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="E5" s="5">
         <v>4</v>
@@ -1567,10 +1567,10 @@
         <v>54</v>
       </c>
       <c r="C6">
-        <v>4801</v>
+        <v>5675</v>
       </c>
       <c r="D6">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="E6" s="5">
         <v>5</v>
@@ -1584,10 +1584,10 @@
         <v>55</v>
       </c>
       <c r="C7">
-        <v>4848</v>
+        <v>5731</v>
       </c>
       <c r="D7">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="E7" s="5">
         <v>4</v>
@@ -1601,10 +1601,10 @@
         <v>56</v>
       </c>
       <c r="C8">
-        <v>4329</v>
+        <v>5665</v>
       </c>
       <c r="D8">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E8" s="5">
         <v>6</v>
@@ -1618,10 +1618,10 @@
         <v>53</v>
       </c>
       <c r="C9">
-        <v>3364</v>
+        <v>3330</v>
       </c>
       <c r="D9">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="E9" s="5">
         <v>3</v>
@@ -1635,10 +1635,10 @@
         <v>54</v>
       </c>
       <c r="C10">
-        <v>2949</v>
+        <v>2990</v>
       </c>
       <c r="D10">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E10" s="5">
         <v>4</v>
@@ -1652,10 +1652,10 @@
         <v>55</v>
       </c>
       <c r="C11">
-        <v>2940</v>
+        <v>2975</v>
       </c>
       <c r="D11">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="E11" s="5">
         <v>4</v>
@@ -1669,13 +1669,13 @@
         <v>56</v>
       </c>
       <c r="C12">
-        <v>2923</v>
+        <v>2990</v>
       </c>
       <c r="D12">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="E12" s="5">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -1686,10 +1686,10 @@
         <v>53</v>
       </c>
       <c r="C13">
-        <v>4687</v>
+        <v>3604</v>
       </c>
       <c r="D13">
-        <v>96</v>
+        <v>71</v>
       </c>
       <c r="E13" s="5">
         <v>4</v>
@@ -1703,10 +1703,10 @@
         <v>54</v>
       </c>
       <c r="C14">
-        <v>4281</v>
+        <v>3271</v>
       </c>
       <c r="D14">
-        <v>91</v>
+        <v>67</v>
       </c>
       <c r="E14" s="5">
         <v>4</v>
@@ -1720,13 +1720,13 @@
         <v>55</v>
       </c>
       <c r="C15">
-        <v>4101</v>
+        <v>3077</v>
       </c>
       <c r="D15">
-        <v>116</v>
+        <v>81</v>
       </c>
       <c r="E15" s="5">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -1737,13 +1737,13 @@
         <v>56</v>
       </c>
       <c r="C16">
-        <v>5325</v>
+        <v>3690</v>
       </c>
       <c r="D16">
-        <v>86</v>
+        <v>58</v>
       </c>
       <c r="E16" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -1754,10 +1754,10 @@
         <v>53</v>
       </c>
       <c r="C17">
-        <v>2995</v>
+        <v>3109</v>
       </c>
       <c r="D17">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E17" s="5">
         <v>6</v>
@@ -1771,10 +1771,10 @@
         <v>54</v>
       </c>
       <c r="C18">
-        <v>2620</v>
+        <v>2729</v>
       </c>
       <c r="D18">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E18" s="5">
         <v>6</v>
@@ -1788,10 +1788,10 @@
         <v>55</v>
       </c>
       <c r="C19">
-        <v>2536</v>
+        <v>2665</v>
       </c>
       <c r="D19">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="E19" s="5">
         <v>7</v>
@@ -1805,10 +1805,10 @@
         <v>56</v>
       </c>
       <c r="C20">
-        <v>2677</v>
+        <v>2922</v>
       </c>
       <c r="D20">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="E20" s="5">
         <v>6</v>
@@ -1862,10 +1862,10 @@
         <v>67</v>
       </c>
       <c r="C5" s="10">
-        <v>265024</v>
+        <v>265203</v>
       </c>
       <c r="D5" s="11">
-        <v>342367</v>
+        <v>342608</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1876,10 +1876,10 @@
         <v>69</v>
       </c>
       <c r="C6" s="10">
-        <v>402906</v>
+        <v>403788</v>
       </c>
       <c r="D6" s="11">
-        <v>529981</v>
+        <v>531163</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1890,10 +1890,10 @@
         <v>71</v>
       </c>
       <c r="C7" s="10">
-        <v>407428</v>
+        <v>407642</v>
       </c>
       <c r="D7" s="11">
-        <v>544449</v>
+        <v>544736</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1904,10 +1904,10 @@
         <v>73</v>
       </c>
       <c r="C8" s="10">
-        <v>383410</v>
+        <v>383500</v>
       </c>
       <c r="D8" s="11">
-        <v>476809</v>
+        <v>476921</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1918,10 +1918,10 @@
         <v>75</v>
       </c>
       <c r="C9" s="10">
-        <v>594748</v>
+        <v>595146</v>
       </c>
       <c r="D9" s="11">
-        <v>746325</v>
+        <v>746846</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1932,10 +1932,10 @@
         <v>77</v>
       </c>
       <c r="C10" s="10">
-        <v>1023684</v>
+        <v>1027312</v>
       </c>
       <c r="D10" s="11">
-        <v>1064159</v>
+        <v>1068056</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1946,10 +1946,10 @@
         <v>79</v>
       </c>
       <c r="C11" s="10">
-        <v>227031</v>
+        <v>227010</v>
       </c>
       <c r="D11" s="11">
-        <v>332600</v>
+        <v>332570</v>
       </c>
     </row>
   </sheetData>
@@ -2255,7 +2255,7 @@
         <v>585</v>
       </c>
       <c r="D23" s="4">
-        <v>0.757</v>
+        <v>0.7559999999999999</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
PAUSED (task190, task193): checkpoint, the positive-control pattern going into checks and the ask repair under way
task190 is putting the positive-control pattern into its document assertions, so an absence check
proves it read the document before it reports nothing found. task193 is working the three devices
its judge found adjudicated by filed documentation, removing the sentences rather than pinning the
sources, which keeps each device standing on the internal inconsistency it was designed around.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017NMcBvUc2Vu9DKDdwmhqo4
</commit_message>
<xml_diff>
--- a/task193/golden/sequence_screen_2027Q1.xlsx
+++ b/task193/golden/sequence_screen_2027Q1.xlsx
@@ -1550,10 +1550,10 @@
         <v>53</v>
       </c>
       <c r="C5">
-        <v>6283</v>
+        <v>5265</v>
       </c>
       <c r="D5">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="E5" s="5">
         <v>4</v>
@@ -1567,10 +1567,10 @@
         <v>54</v>
       </c>
       <c r="C6">
-        <v>5657</v>
+        <v>4783</v>
       </c>
       <c r="D6">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="E6" s="5">
         <v>5</v>
@@ -1584,10 +1584,10 @@
         <v>55</v>
       </c>
       <c r="C7">
-        <v>5724</v>
+        <v>4877</v>
       </c>
       <c r="D7">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="E7" s="5">
         <v>4</v>
@@ -1601,10 +1601,10 @@
         <v>56</v>
       </c>
       <c r="C8">
-        <v>5639</v>
+        <v>4647</v>
       </c>
       <c r="D8">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="E8" s="5">
         <v>6</v>
@@ -1618,10 +1618,10 @@
         <v>53</v>
       </c>
       <c r="C9">
-        <v>3330</v>
+        <v>4554</v>
       </c>
       <c r="D9">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="E9" s="5">
         <v>3</v>
@@ -1635,10 +1635,10 @@
         <v>54</v>
       </c>
       <c r="C10">
-        <v>2981</v>
+        <v>4079</v>
       </c>
       <c r="D10">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="E10" s="5">
         <v>4</v>
@@ -1652,10 +1652,10 @@
         <v>55</v>
       </c>
       <c r="C11">
-        <v>3025</v>
+        <v>4011</v>
       </c>
       <c r="D11">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="E11" s="5">
         <v>4</v>
@@ -1669,10 +1669,10 @@
         <v>56</v>
       </c>
       <c r="C12">
-        <v>3159</v>
+        <v>4380</v>
       </c>
       <c r="D12">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="E12" s="5">
         <v>6</v>
@@ -1686,10 +1686,10 @@
         <v>53</v>
       </c>
       <c r="C13">
-        <v>3597</v>
+        <v>3777</v>
       </c>
       <c r="D13">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E13" s="5">
         <v>4</v>
@@ -1703,10 +1703,10 @@
         <v>54</v>
       </c>
       <c r="C14">
-        <v>3258</v>
+        <v>3316</v>
       </c>
       <c r="D14">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E14" s="5">
         <v>4</v>
@@ -1720,10 +1720,10 @@
         <v>55</v>
       </c>
       <c r="C15">
-        <v>3019</v>
+        <v>3123</v>
       </c>
       <c r="D15">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="E15" s="5">
         <v>5</v>
@@ -1737,10 +1737,10 @@
         <v>56</v>
       </c>
       <c r="C16">
-        <v>3473</v>
+        <v>3613</v>
       </c>
       <c r="D16">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="E16" s="5">
         <v>4</v>
@@ -1754,10 +1754,10 @@
         <v>53</v>
       </c>
       <c r="C17">
-        <v>3113</v>
+        <v>2719</v>
       </c>
       <c r="D17">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E17" s="5">
         <v>6</v>
@@ -1771,13 +1771,13 @@
         <v>54</v>
       </c>
       <c r="C18">
-        <v>2715</v>
+        <v>2434</v>
       </c>
       <c r="D18">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="E18" s="5">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -1788,10 +1788,10 @@
         <v>55</v>
       </c>
       <c r="C19">
-        <v>2673</v>
+        <v>2419</v>
       </c>
       <c r="D19">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E19" s="5">
         <v>7</v>
@@ -1805,10 +1805,10 @@
         <v>56</v>
       </c>
       <c r="C20">
-        <v>3005</v>
+        <v>2633</v>
       </c>
       <c r="D20">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E20" s="5">
         <v>6</v>
@@ -1862,10 +1862,10 @@
         <v>67</v>
       </c>
       <c r="C5" s="10">
-        <v>282252</v>
+        <v>281932</v>
       </c>
       <c r="D5" s="11">
-        <v>353865</v>
+        <v>353483</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1876,10 +1876,10 @@
         <v>69</v>
       </c>
       <c r="C6" s="10">
-        <v>503166.5</v>
+        <v>504333.5</v>
       </c>
       <c r="D6" s="11">
-        <v>632763</v>
+        <v>634199</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1890,10 +1890,10 @@
         <v>71</v>
       </c>
       <c r="C7" s="10">
-        <v>434820</v>
+        <v>434434</v>
       </c>
       <c r="D7" s="11">
-        <v>558081</v>
+        <v>557585</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1904,10 +1904,10 @@
         <v>73</v>
       </c>
       <c r="C8" s="10">
-        <v>204605</v>
+        <v>204690</v>
       </c>
       <c r="D8" s="11">
-        <v>304072</v>
+        <v>304182</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1918,10 +1918,10 @@
         <v>75</v>
       </c>
       <c r="C9" s="10">
-        <v>627178</v>
+        <v>626840</v>
       </c>
       <c r="D9" s="11">
-        <v>770812</v>
+        <v>770394</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1932,10 +1932,10 @@
         <v>77</v>
       </c>
       <c r="C10" s="10">
-        <v>1090114</v>
+        <v>1088808</v>
       </c>
       <c r="D10" s="11">
-        <v>1132391</v>
+        <v>1131025</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1946,10 +1946,10 @@
         <v>79</v>
       </c>
       <c r="C11" s="10">
-        <v>121348.5</v>
+        <v>120991.5</v>
       </c>
       <c r="D11" s="11">
-        <v>179474</v>
+        <v>178946</v>
       </c>
     </row>
   </sheetData>
@@ -2000,10 +2000,10 @@
         <v>86</v>
       </c>
       <c r="C5">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D5" s="4">
-        <v>0.705</v>
+        <v>0.7040000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -2014,10 +2014,10 @@
         <v>87</v>
       </c>
       <c r="C6">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="D6" s="4">
-        <v>0.6890000000000001</v>
+        <v>0.6870000000000001</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -2028,10 +2028,10 @@
         <v>88</v>
       </c>
       <c r="C7">
-        <v>1089</v>
+        <v>1085</v>
       </c>
       <c r="D7" s="4">
-        <v>0.7979999999999999</v>
+        <v>0.797</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -2042,10 +2042,10 @@
         <v>89</v>
       </c>
       <c r="C8">
-        <v>680</v>
+        <v>679</v>
       </c>
       <c r="D8" s="4">
-        <v>0.8029999999999999</v>
+        <v>0.804</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -2056,10 +2056,10 @@
         <v>86</v>
       </c>
       <c r="C9">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="D9" s="4">
-        <v>0.6890000000000001</v>
+        <v>0.6859999999999999</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -2070,10 +2070,10 @@
         <v>87</v>
       </c>
       <c r="C10">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="D10" s="4">
-        <v>0.696</v>
+        <v>0.695</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -2084,10 +2084,10 @@
         <v>88</v>
       </c>
       <c r="C11">
-        <v>876</v>
+        <v>864</v>
       </c>
       <c r="D11" s="4">
-        <v>0.7829999999999999</v>
+        <v>0.7809999999999999</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -2098,10 +2098,10 @@
         <v>89</v>
       </c>
       <c r="C12">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="D12" s="4">
-        <v>0.772</v>
+        <v>0.773</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -2112,10 +2112,10 @@
         <v>86</v>
       </c>
       <c r="C13">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D13" s="4">
-        <v>0.6920000000000001</v>
+        <v>0.696</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -2126,10 +2126,10 @@
         <v>87</v>
       </c>
       <c r="C14">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D14" s="4">
-        <v>0.6920000000000001</v>
+        <v>0.6909999999999999</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -2140,10 +2140,10 @@
         <v>88</v>
       </c>
       <c r="C15">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D15" s="4">
-        <v>0.773</v>
+        <v>0.774</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -2168,10 +2168,10 @@
         <v>86</v>
       </c>
       <c r="C17">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D17" s="4">
-        <v>0.695</v>
+        <v>0.6970000000000001</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -2182,10 +2182,10 @@
         <v>87</v>
       </c>
       <c r="C18">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="D18" s="4">
-        <v>0.7609999999999999</v>
+        <v>0.762</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -2196,10 +2196,10 @@
         <v>88</v>
       </c>
       <c r="C19">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="D19" s="4">
-        <v>0.7659999999999999</v>
+        <v>0.767</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -2213,7 +2213,7 @@
         <v>362</v>
       </c>
       <c r="D20" s="4">
-        <v>0.804</v>
+        <v>0.7979999999999999</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -2224,10 +2224,10 @@
         <v>86</v>
       </c>
       <c r="C21">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D21" s="4">
-        <v>0.7190000000000001</v>
+        <v>0.721</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -2241,7 +2241,7 @@
         <v>562</v>
       </c>
       <c r="D22" s="4">
-        <v>0.7170000000000001</v>
+        <v>0.721</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -2252,10 +2252,10 @@
         <v>88</v>
       </c>
       <c r="C23">
-        <v>867</v>
+        <v>879</v>
       </c>
       <c r="D23" s="4">
-        <v>0.767</v>
+        <v>0.769</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -2266,10 +2266,10 @@
         <v>89</v>
       </c>
       <c r="C24">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="D24" s="4">
-        <v>0.805</v>
+        <v>0.8070000000000001</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>